<commit_message>
updated file for system scenarios
</commit_message>
<xml_diff>
--- a/SystemTesting.xlsx
+++ b/SystemTesting.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Downloads\excel Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D15BCFC2-00CA-4EA3-BB6B-1C7158D3F938}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C35596DC-0A00-422E-B8A9-6F5C92B97D50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{76F801B5-FC76-4A46-A4A9-5DE17DE76C26}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" activeTab="6" xr2:uid="{76F801B5-FC76-4A46-A4A9-5DE17DE76C26}"/>
   </bookViews>
   <sheets>
     <sheet name="LOGIN_REGISTER" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="121">
   <si>
     <t>APPLICATION_NAME</t>
   </si>
@@ -69,21 +69,6 @@
     <t>LOGIN / REGISTER</t>
   </si>
   <si>
-    <t>TO VERIFY EXISTING USER CAN LOGIN USING VALID CREDENTIALS</t>
-  </si>
-  <si>
-    <t>TO VERIFY SYSTEM SHOWS ERROR MESSAGE WHEN INVALID LOGIN CREDENTIALS ARE ENTERED</t>
-  </si>
-  <si>
-    <t>TO VERIFY USER CAN RESET PASSWORD USING FORGOT PASSWORD OPTION</t>
-  </si>
-  <si>
-    <t>TO VERIFY USER CAN LOGOUT SUCCESSFULLY FROM INSTAGRAM</t>
-  </si>
-  <si>
-    <t>TO VERIFY USER SESSION EXPIRES AFTER LONG INACTIVITY</t>
-  </si>
-  <si>
     <t>INSTA_LOGIN_001</t>
   </si>
   <si>
@@ -96,33 +81,15 @@
     <t>INSTA_LOGIN_004</t>
   </si>
   <si>
-    <t>INSTA_LOGIN_005</t>
-  </si>
-  <si>
-    <t>INSTA_LOGIN_006</t>
-  </si>
-  <si>
     <t>HOME FEED</t>
   </si>
   <si>
-    <t>TO VERIFY USER CAN VIEW POSTS FROM FOLLOWED ACCOUNTS IN HOME FEED</t>
-  </si>
-  <si>
-    <t>TO VERIFY NEW POSTS FROM FOLLOWED USERS APPEAR IN HOME FEED</t>
-  </si>
-  <si>
-    <t>TO VERIFY USER CAN VIEW STORIES FROM HOME FEED STORY SECTION</t>
-  </si>
-  <si>
     <t>LOGIN → HOME FEED → STORY SECTION → SELECT STORY → VIEW STORY</t>
   </si>
   <si>
     <t>LOGIN → HOME FEED → SELECT POST → CLICK USERNAME → OPEN USER PROFILE</t>
   </si>
   <si>
-    <t>TO VERIFY USER CAN REFRESH HOME FEED TO LOAD NEW POSTS</t>
-  </si>
-  <si>
     <t>INSTA_HOME_001</t>
   </si>
   <si>
@@ -138,9 +105,6 @@
     <t>INSTA_HOME_005</t>
   </si>
   <si>
-    <t>INSTA_HOME_006</t>
-  </si>
-  <si>
     <t>POST CREATION</t>
   </si>
   <si>
@@ -159,21 +123,9 @@
     <t>INSTA_POSTCREATION_004</t>
   </si>
   <si>
-    <t>INSTA_POSTCREATION_005</t>
-  </si>
-  <si>
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>TO VERIFY POST OWNER RECEIVES NOTIFICATION WHEN SOMEONE LIKES THEIR POST</t>
-  </si>
-  <si>
-    <t>TO VERIFY POST OWNER RECEIVES NOTIFICATION WHEN SOMEONE COMMENTS ON THEIR POST</t>
-  </si>
-  <si>
-    <t>LOGIN → SELECT POST → ENTER EMPTY COMMENT → ERROR MESSAGE DISPLAYED</t>
-  </si>
-  <si>
     <t>LIKE / COMMENT MODULE</t>
   </si>
   <si>
@@ -189,12 +141,6 @@
     <t>INSTA_LIKE_004</t>
   </si>
   <si>
-    <t>INSTA_LIKE_005</t>
-  </si>
-  <si>
-    <t>INSTA_LIKE_006</t>
-  </si>
-  <si>
     <t>FOLLOW / UNFOLLOW MODULE</t>
   </si>
   <si>
@@ -207,9 +153,6 @@
     <t>TO VERIFY USER CAN UNFOLLOW A FOLLOWED ACCOUNT</t>
   </si>
   <si>
-    <t>LOGIN → OPEN FOLLOWED USER PROFILE → CLICK UNFOLLOW → USER REMOVED FROM FOLLOWING LIST</t>
-  </si>
-  <si>
     <t>TO VERIFY USER RECEIVES NOTIFICATION WHEN SOMEONE FOLLOWS THEM</t>
   </si>
   <si>
@@ -234,66 +177,12 @@
     <t>SEARCH MODULE</t>
   </si>
   <si>
-    <t>TO VERIFY USER CAN SEARCH AN ACCOUNT USING USERNAME</t>
-  </si>
-  <si>
-    <t>LOGIN → SEARCH ICON → ENTER USERNAME → FETCH RESULTS → DISPLAY USER PROFILE</t>
-  </si>
-  <si>
-    <t>TO VERIFY USER CAN SEARCH POSTS USING HASHTAGS</t>
-  </si>
-  <si>
-    <t>LOGIN → SEARCH SECTION → ENTER HASHTAG → FETCH POSTS → DISPLAY RELATED POSTS</t>
-  </si>
-  <si>
-    <t>TO VERIFY USER CAN SEARCH REELS USING KEYWORDS</t>
-  </si>
-  <si>
-    <t>LOGIN → SEARCH BAR → ENTER KEYWORD → FETCH REELS → DISPLAY REELS RESULTS</t>
-  </si>
-  <si>
-    <t>TO VERIFY SEARCH RESULTS DISPLAY MATCHING USERS</t>
-  </si>
-  <si>
-    <t>LOGIN → SEARCH BAR → ENTER USERNAME → SEARCH SERVICE → DISPLAY MATCHING USERS</t>
-  </si>
-  <si>
-    <t>TO VERIFY USER CAN OPEN PROFILE FROM SEARCH RESULTS</t>
-  </si>
-  <si>
-    <t>LOGIN → SEARCH USER → SELECT PROFILE → OPEN USER PROFILE PAGE</t>
-  </si>
-  <si>
     <t>TO VERIFY USER CAN FOLLOW ACCOUNT FROM SEARCH RESULTS</t>
   </si>
   <si>
-    <t>LOGIN → SEARCH USER → OPEN PROFILE → CLICK FOLLOW</t>
-  </si>
-  <si>
-    <t>TO VERIFY SYSTEM SHOWS RECENT SEARCH HISTORY</t>
-  </si>
-  <si>
-    <t>LOGIN → SEARCH SECTION → VIEW RECENT SEARCHES</t>
-  </si>
-  <si>
-    <t>TO VERIFY USER CAN CLEAR SEARCH HISTORY</t>
-  </si>
-  <si>
     <t>LOGIN → SEARCH SECTION → VIEW SEARCH HISTORY → CLEAR HISTORY</t>
   </si>
   <si>
-    <t>TO VERIFY SYSTEM SHOWS TRENDING POSTS IN SEARCH PAGE</t>
-  </si>
-  <si>
-    <t>LOGIN → SEARCH PAGE → FETCH TRENDING CONTENT → DISPLAY TRENDING POSTS</t>
-  </si>
-  <si>
-    <t>TO VERIFY SYSTEM SHOWS ERROR OR EMPTY RESULT WHEN NO MATCHING CONTENT IS FOUND</t>
-  </si>
-  <si>
-    <t>LOGIN → SEARCH BAR → ENTER INVALID KEYWORD → DISPLAY NO RESULTS MESSAGE</t>
-  </si>
-  <si>
     <t>INSTA_SEARCH_001</t>
   </si>
   <si>
@@ -309,75 +198,12 @@
     <t>INSTA_SEARCH_005</t>
   </si>
   <si>
-    <t>INSTA_SEARCH_006</t>
-  </si>
-  <si>
-    <t>INSTA_SEARCH_007</t>
-  </si>
-  <si>
-    <t>INSTA_SEARCH_008</t>
-  </si>
-  <si>
-    <t>INSTA_SEARCH_009</t>
-  </si>
-  <si>
-    <t>INSTA_SEARCH_010</t>
-  </si>
-  <si>
     <t>STORY MODULE</t>
   </si>
   <si>
-    <t>TO VERIFY USER CAN CREATE AND UPLOAD A STORY SUCCESSFULLY</t>
-  </si>
-  <si>
-    <t>LOGIN → HOME PAGE → CREATE STORY → CAPTURE/UPLOAD MEDIA → POST STORY → STORY DISPLAYED</t>
-  </si>
-  <si>
-    <t>TO VERIFY FOLLOWERS CAN VIEW USER STORY</t>
-  </si>
-  <si>
-    <t>LOGIN → USER A UPLOADS STORY → USER B HOME FEED → CLICK STORY → VIEW STORY</t>
-  </si>
-  <si>
-    <t>TO VERIFY STORY DISAPPEARS AFTER 24 HOURS</t>
-  </si>
-  <si>
-    <t>LOGIN → CREATE STORY → STORY DISPLAYED → 24 HOURS COMPLETED → STORY REMOVED</t>
-  </si>
-  <si>
-    <t>TO VERIFY USER CAN VIEW MULTIPLE STORIES FROM DIFFERENT USERS</t>
-  </si>
-  <si>
-    <t>LOGIN → HOME PAGE → STORY SECTION → SELECT STORIES → VIEW STORIES SEQUENTIALLY</t>
-  </si>
-  <si>
-    <t>TO VERIFY USER CAN REPLY TO A STORY</t>
-  </si>
-  <si>
-    <t>LOGIN → VIEW STORY → ENTER MESSAGE → SEND REPLY → MESSAGE SENT TO STORY OWNER</t>
-  </si>
-  <si>
-    <t>TO VERIFY STORY OWNER RECEIVES NOTIFICATION FOR STORY REPLIES</t>
-  </si>
-  <si>
-    <t>LOGIN → USER A POSTS STORY → USER B REPLIES → NOTIFICATION SENT TO USER A</t>
-  </si>
-  <si>
     <t>TO VERIFY USER CAN DELETE THEIR STORY</t>
   </si>
   <si>
-    <t>LOGIN → CREATE STORY → OPEN STORY OPTIONS → DELETE STORY</t>
-  </si>
-  <si>
-    <t>TO VERIFY USER CAN SEE LIST OF USERS WHO VIEWED THEIR STORY</t>
-  </si>
-  <si>
-    <t>LOGIN → POST STORY → VIEW STORY INSIGHTS → DISPLAY VIEWERS LIST</t>
-  </si>
-  <si>
-    <t>TO VERIFY USER CAN SHARE POST TO STORY</t>
-  </si>
-  <si>
     <t>LOGIN → OPEN POST → SHARE → ADD TO STORY → STORY POSTED</t>
   </si>
   <si>
@@ -408,39 +234,18 @@
     <t>INSTA_STORY_007</t>
   </si>
   <si>
-    <t>INSTA_STORY_008</t>
-  </si>
-  <si>
-    <t>INSTA_STORY_009</t>
-  </si>
-  <si>
-    <t>INSTA_STORY_010</t>
-  </si>
-  <si>
     <t>REGISTER → ENTER USER DETAILS → EMAIL/OTP VERIFICATION → ACCOUNT CREATED → LOGIN → HOME FEED</t>
   </si>
   <si>
     <t>LOGIN PAGE → ENTER USERNAME/EMAIL/MOBILE AND PASSWORD → LOGIN → HOME FEED DISPLAYED</t>
   </si>
   <si>
-    <t>LOGIN PAGE → ENTER INVALID CREDENTIALS → CLICK LOGIN → ERROR MESSAGE DISPLAYED</t>
-  </si>
-  <si>
-    <t>LOGIN PAGE → CLICK FORGOT PASSWORD → ENTER EMAIL/MOBILE → OTP VERIFICATION → RESET PASSWORD → LOGIN SUCCESS</t>
-  </si>
-  <si>
     <t>LOGIN → HOME FEED → PROFILE → LOGOUT → REDIRECT TO LOGIN PAGE</t>
   </si>
   <si>
     <t>LOGIN → HOME FEED → POSTS FROM FOLLOWED USERS DISPLAYED</t>
   </si>
   <si>
-    <t>LOGIN → FOLLOW USERS → USER POSTS CONTENT → REFRESH HOME FEED → NEW POST DISPLAYED</t>
-  </si>
-  <si>
-    <t>TO VERIFY USER CAN NAVIGATE TO USER PROFILE FROM A POST</t>
-  </si>
-  <si>
     <t>LOGIN → HOME FEED → PULL TO REFRESH → NEW POSTS DISPLAYED</t>
   </si>
   <si>
@@ -450,63 +255,21 @@
     <t>TO VERIFY USER CAN EDIT POST DETAILS AFTER POST CREATION</t>
   </si>
   <si>
-    <t>TO VERIFY NEW USER CAN REGISTER AND ACCESS INSTAGRAM SUCCESSFULLY</t>
-  </si>
-  <si>
-    <t>LOGIN → USE APPLICATION → USER INACTIVE FOR LONG TIME → SESSION EXPIRES → REDIRECT TO LOGIN PAGE</t>
-  </si>
-  <si>
     <t>TO VERIFY USER CAN VIEW AND INTERACT WITH POSTS FROM HOME FEED</t>
   </si>
   <si>
-    <t>LOGIN → HOME FEED → SELECT POST → LIKE / COMMENT / SAVE / SHARE POST</t>
-  </si>
-  <si>
-    <t>TO VERIFY USER CAN CREATE AND PUBLISH A POST USING AVAILABLE POST FEATURES</t>
-  </si>
-  <si>
     <t>LOGIN → CREATE POST → SELECT PHOTO/VIDEO → EDIT MEDIA → ADD CAPTION / TAG USERS / ADD LOCATION → PUBLISH POST → POST DISPLAYED IN PROFILE AND FOLLOWERS FEED</t>
   </si>
   <si>
     <t>LOGIN → CREATE POST → PUBLISH POST → SHARE POST → ADD TO STORY → STORY DISPLAYED</t>
   </si>
   <si>
-    <t>LOGIN → CREATE POST → PUBLISH POST → OPEN POST OPTIONS → EDIT CAPTION / LOCATION → SAVE CHANGES</t>
-  </si>
-  <si>
     <t>LOGIN → CREATE POST → PUBLISH POST → OPEN POST OPTIONS → DELETE POST → POST REMOVED FROM PROFILE</t>
   </si>
   <si>
-    <t>TO VERIFY SYSTEM SHOWS ERROR MESSAGE IF USER TRIES TO POST WITHOUT SELECTING MEDIA</t>
-  </si>
-  <si>
-    <t>LOGIN → CREATE POST → NO MEDIA SELECTED → TRY TO PUBLISH POST → ERROR MESSAGE DISPLAYED</t>
-  </si>
-  <si>
-    <t>TO VERIFY USER CAN LIKE AND UNLIKE A POST FROM HOME FEED</t>
-  </si>
-  <si>
-    <t>LOGIN → HOME FEED → SELECT POST → LIKE POST → UNLIKE POST</t>
-  </si>
-  <si>
-    <t>LOGIN → USER A POSTS CONTENT → USER B LIKES POST → NOTIFICATION DISPLAYED TO USER A</t>
-  </si>
-  <si>
-    <t>TO VERIFY USER CAN ADD AND MANAGE COMMENTS ON A POST</t>
-  </si>
-  <si>
     <t>LOGIN → HOME FEED → SELECT POST → ADD COMMENT → EDIT / DELETE COMMENT</t>
   </si>
   <si>
-    <t>LOGIN → USER A POSTS CONTENT → USER B COMMENTS → NOTIFICATION DISPLAYED TO USER A</t>
-  </si>
-  <si>
-    <t>TO VERIFY SYSTEM SHOWS ERROR MESSAGE WHEN USER TRIES TO SUBMIT EMPTY COMMENT</t>
-  </si>
-  <si>
-    <t>TO VERIFY LIKE AND COMMENT ACTIONS ARE REFLECTED FOR OTHER USERS</t>
-  </si>
-  <si>
     <t>LOGIN → USER A POSTS CONTENT → USER B LIKES / COMMENTS → USER A REFRESHES FEED → UPDATE DISPLAYED</t>
   </si>
   <si>
@@ -525,10 +288,121 @@
     <t>LOGIN → USER A FOLLOWS USER B → NOTIFICATION DISPLAYED TO USER B</t>
   </si>
   <si>
-    <t>TO VERIFY USER CAN VIEW LIST OF FOLLOWERS AND FOLLOWING USERS</t>
-  </si>
-  <si>
     <t>LOGIN → OPEN PROFILE → VIEW FOLLOWERS / FOLLOWING LIST</t>
+  </si>
+  <si>
+    <t>TO VERIFY NEW USER CAN REGISTER AND ACCESS INSTAGRAM</t>
+  </si>
+  <si>
+    <t>TO VERIFY EXISTING USER CAN LOGIN AND ACCESS INSTAGRAM</t>
+  </si>
+  <si>
+    <t>TO VERIFY USER CAN RESET PASSWORD AND LOGIN TO INSTAGRAM</t>
+  </si>
+  <si>
+    <t>LOGIN PAGE → CLICK FORGOT PASSWORD → ENTER EMAIL/MOBILE → OTP VERIFICATION → RESET PASSWORD → LOGIN → HOME FEED</t>
+  </si>
+  <si>
+    <t>TO VERIFY USER CAN LOGOUT FROM INSTAGRAM</t>
+  </si>
+  <si>
+    <t>TO VERIFY USER CAN ACCESS AND VIEW CONTENT IN HOME FEED</t>
+  </si>
+  <si>
+    <t>LOGIN → HOME FEED → SELECT POST → LIKE / COMMENT / SAVE / SHARE</t>
+  </si>
+  <si>
+    <t>TO VERIFY USER CAN VIEW STORIES FROM HOME FEED</t>
+  </si>
+  <si>
+    <t>TO VERIFY USER CAN NAVIGATE TO USER PROFILE FROM HOME FEED</t>
+  </si>
+  <si>
+    <t>TO VERIFY USER CAN REFRESH HOME FEED TO LOAD NEW CONTENT</t>
+  </si>
+  <si>
+    <t>TO VERIFY USER CAN CREATE AND PUBLISH A POST USING AVAILABLE FEATURES</t>
+  </si>
+  <si>
+    <t>LOGIN → CREATE POST → PUBLISH POST → OPEN POST OPTIONS → EDIT POST DETAILS → SAVE CHANGES</t>
+  </si>
+  <si>
+    <t>TO VERIFY USER CAN INTERACT WITH A POST USING LIKE AND COMMENT FEATURES</t>
+  </si>
+  <si>
+    <t>LOGIN → HOME FEED → SELECT POST → LIKE POST → ADD COMMENT</t>
+  </si>
+  <si>
+    <t>TO VERIFY POST OWNER RECEIVES NOTIFICATION WHEN SOMEONE INTERACTS WITH THEIR POST</t>
+  </si>
+  <si>
+    <t>LOGIN → USER A POSTS CONTENT → USER B LIKES / COMMENTS → NOTIFICATION DISPLAYED TO USER A</t>
+  </si>
+  <si>
+    <t>TO VERIFY USER CAN MANAGE COMMENTS ON A POST</t>
+  </si>
+  <si>
+    <t>TO VERIFY POST INTERACTIONS ARE REFLECTED FOR OTHER USERS</t>
+  </si>
+  <si>
+    <t>LOGIN → OPEN USER PROFILE → CLICK UNFOLLOW → USER REMOVED FROM FOLLOWING LIST</t>
+  </si>
+  <si>
+    <t>TO VERIFY USER CAN VIEW FOLLOWERS AND FOLLOWING LIST</t>
+  </si>
+  <si>
+    <t>TO VERIFY USER CAN SEARCH AND VIEW CONTENT ON INSTAGRAM</t>
+  </si>
+  <si>
+    <t>LOGIN → SEARCH → ENTER USERNAME / HASHTAG / KEYWORD → SEARCH RESULTS DISPLAYED</t>
+  </si>
+  <si>
+    <t>TO VERIFY USER CAN OPEN PROFILE OR CONTENT FROM SEARCH RESULTS</t>
+  </si>
+  <si>
+    <t>LOGIN → SEARCH → ENTER KEYWORD → VIEW RESULTS → OPEN USER PROFILE / POST / REEL</t>
+  </si>
+  <si>
+    <t>LOGIN → SEARCH USER → OPEN USER PROFILE → CLICK FOLLOW</t>
+  </si>
+  <si>
+    <t>TO VERIFY SYSTEM DISPLAYS TRENDING CONTENT IN SEARCH PAGE</t>
+  </si>
+  <si>
+    <t>LOGIN → OPEN SEARCH PAGE → TRENDING POSTS / REELS DISPLAYED</t>
+  </si>
+  <si>
+    <t>TO VERIFY USER CAN VIEW AND MANAGE SEARCH HISTORY</t>
+  </si>
+  <si>
+    <t>TO VERIFY USER CAN CREATE AND SHARE A STORY</t>
+  </si>
+  <si>
+    <t>LOGIN → HOME PAGE → CREATE STORY → CAPTURE / UPLOAD MEDIA → POST STORY → STORY DISPLAYED</t>
+  </si>
+  <si>
+    <t>TO VERIFY USERS CAN VIEW STORIES FROM FOLLOWED ACCOUNTS</t>
+  </si>
+  <si>
+    <t>LOGIN → HOME PAGE → STORY SECTION → SELECT STORY → VIEW STORY</t>
+  </si>
+  <si>
+    <t>TO VERIFY USER CAN INTERACT WITH A STORY</t>
+  </si>
+  <si>
+    <t>LOGIN → VIEW STORY → SEND STORY REPLY → MESSAGE SENT TO STORY OWNER</t>
+  </si>
+  <si>
+    <t>TO VERIFY USER CAN VIEW STORY INSIGHTS</t>
+  </si>
+  <si>
+    <t>LOGIN → POST STORY → OPEN STORY → VIEW STORY VIEWERS LIST</t>
+  </si>
+  <si>
+    <t>LOGIN → POST STORY → OPEN STORY OPTIONS → DELETE STORY</t>
+  </si>
+  <si>
+    <t>TO VERIFY USER CAN SHARE A POST TO STORY</t>
   </si>
 </sst>
 </file>
@@ -593,12 +467,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -611,13 +482,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -967,101 +838,89 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>125</v>
+      <c r="A6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>126</v>
+      <c r="A7" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" s="6" t="s">
+      <c r="A8" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="6" t="s">
+      <c r="B8" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A11" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>137</v>
-      </c>
+      <c r="B9" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="9"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="9"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
+      <c r="A13" s="6"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="7"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
+      <c r="A15" s="5"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1092,7 +951,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1104,101 +963,95 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>130</v>
+      <c r="A6" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>131</v>
+      <c r="A7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>139</v>
+      <c r="A8" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>24</v>
+      <c r="A9" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A11" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>133</v>
-      </c>
+      <c r="A10" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="9"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="9"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
+      <c r="A13" s="6"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="7"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
+      <c r="A15" s="5"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1229,7 +1082,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1242,99 +1095,93 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>141</v>
+      <c r="A6" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>142</v>
+      <c r="A7" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>143</v>
+      <c r="A8" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>146</v>
-      </c>
+      <c r="A9" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" s="9"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="9"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="9"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
+      <c r="A13" s="6"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="9"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
+      <c r="A14" s="6"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="9"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
+      <c r="A15" s="6"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1365,7 +1212,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1377,101 +1224,89 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>148</v>
+    <row r="6" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>149</v>
+      <c r="A7" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>151</v>
+      <c r="A8" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A11" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>155</v>
-      </c>
+      <c r="A9" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="9"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="9"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
+      <c r="A13" s="6"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="9"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
+      <c r="A14" s="6"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="9"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
+      <c r="A15" s="6"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
@@ -1508,7 +1343,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1520,101 +1355,101 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A6" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>157</v>
+      <c r="A6" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>53</v>
+      <c r="A7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>55</v>
+      <c r="A8" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A9" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>159</v>
+      <c r="A9" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A10" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A11" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>162</v>
+      <c r="A10" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="9"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="9"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
+      <c r="A13" s="6"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="9"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
+      <c r="A14" s="6"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="9"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
+      <c r="A15" s="6"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1645,7 +1480,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1657,125 +1492,95 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>65</v>
+      <c r="A6" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>71</v>
+      <c r="A7" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>73</v>
+      <c r="A10" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>75</v>
-      </c>
+      <c r="A11" s="7"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>77</v>
-      </c>
+      <c r="A12" s="7"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A14" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A15" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>83</v>
-      </c>
+      <c r="A13" s="7"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="7"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="7"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1806,7 +1611,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1818,125 +1623,107 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A8" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
+    </row>
+    <row r="9" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>104</v>
-      </c>
     </row>
     <row r="11" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>106</v>
+      <c r="C11" s="5" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A12" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A13" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A14" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A15" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>114</v>
-      </c>
+      <c r="A12" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="3"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="3"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="3"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>